<commit_message>
Changes made in NSTP flow of PC
</commit_message>
<xml_diff>
--- a/pages/NB/STPTestData.xlsx
+++ b/pages/NB/STPTestData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\pages\NB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6539FA25-1C5E-4FF4-9762-9FB49C12EB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0C3195C-BABA-4A2E-9818-EDF9F8381038}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{45C1E7C0-1AF2-45CB-BEA8-DD612E61CE1D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="189">
   <si>
     <t>RegNo</t>
   </si>
@@ -550,6 +550,57 @@
   </si>
   <si>
     <t>NSTP</t>
+  </si>
+  <si>
+    <t>SAB5331D</t>
+  </si>
+  <si>
+    <t>971013-12-5147</t>
+  </si>
+  <si>
+    <t>BDJ1366</t>
+  </si>
+  <si>
+    <t>680823-02-5391</t>
+  </si>
+  <si>
+    <t>STP</t>
+  </si>
+  <si>
+    <t>JPE2818</t>
+  </si>
+  <si>
+    <t>030304-06-0561</t>
+  </si>
+  <si>
+    <t>VDB802</t>
+  </si>
+  <si>
+    <t>030324-01-1003</t>
+  </si>
+  <si>
+    <t>WJM8246</t>
+  </si>
+  <si>
+    <t>801122-10-5469</t>
+  </si>
+  <si>
+    <t>WWV358</t>
+  </si>
+  <si>
+    <t>640705-10-7234</t>
+  </si>
+  <si>
+    <t>BGN2294</t>
+  </si>
+  <si>
+    <t>690114-10-5531</t>
+  </si>
+  <si>
+    <t>PCE2215</t>
+  </si>
+  <si>
+    <t>740409-02-6526</t>
   </si>
 </sst>
 </file>
@@ -666,7 +717,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -747,42 +798,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -823,16 +843,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1152,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{689C8A9F-98AE-49F8-89B3-BABBB35DE82F}">
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.36328125" customWidth="1"/>
@@ -1160,12 +1176,12 @@
     <col min="3" max="3" width="13.453125" customWidth="1"/>
     <col min="5" max="5" width="14.08984375" customWidth="1"/>
     <col min="6" max="6" width="18.26953125" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="10" max="10" width="15.36328125" customWidth="1"/>
-    <col min="11" max="11" width="14.7265625" customWidth="1"/>
+    <col min="10" max="10" width="9.08984375" customWidth="1"/>
+    <col min="11" max="11" width="15.36328125" customWidth="1"/>
+    <col min="12" max="12" width="14.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1178,22 +1194,25 @@
       <c r="E1" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="I1" s="26" t="s">
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="26"/>
+      <c r="J1" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="6"/>
+      <c r="C2" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="E2" s="11" t="s">
         <v>89</v>
       </c>
@@ -1203,20 +1222,20 @@
       <c r="G2" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="H2" s="29" t="s">
+      <c r="H2" t="s">
         <v>171</v>
       </c>
-      <c r="I2" s="16" t="s">
+      <c r="J2" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="J2" s="16" t="s">
+      <c r="K2" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="L2" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1233,17 +1252,17 @@
       <c r="G3" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="J3" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="K3" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="K3" s="18" t="s">
+      <c r="L3" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
@@ -1260,17 +1279,17 @@
       <c r="G4" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="J4" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="K4" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="K4" s="18" t="s">
+      <c r="L4" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -1289,17 +1308,17 @@
       <c r="G5" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="J5" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="K5" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="K5" s="18" t="s">
+      <c r="L5" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -1318,17 +1337,17 @@
       <c r="G6" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="J6" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="J6" s="16" t="s">
+      <c r="K6" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="K6" s="18" t="s">
+      <c r="L6" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="24" t="s">
         <v>12</v>
       </c>
@@ -1347,17 +1366,17 @@
       <c r="G7" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I7" s="17" t="s">
+      <c r="J7" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="J7" s="17" t="s">
+      <c r="K7" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="K7" s="19" t="s">
+      <c r="L7" s="19" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="24" t="s">
         <v>14</v>
       </c>
@@ -1376,17 +1395,17 @@
       <c r="G8" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I8" s="16" t="s">
+      <c r="J8" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="J8" s="16" t="s">
+      <c r="K8" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="K8" s="18" t="s">
+      <c r="L8" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -1405,17 +1424,17 @@
       <c r="G9" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="J9" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="J9" s="16" t="s">
+      <c r="K9" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="K9" s="18" t="s">
+      <c r="L9" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>18</v>
       </c>
@@ -1434,17 +1453,17 @@
       <c r="G10" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I10" s="16" t="s">
+      <c r="J10" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="J10" s="16" t="s">
+      <c r="K10" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="K10" s="18" t="s">
+      <c r="L10" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>21</v>
       </c>
@@ -1463,17 +1482,17 @@
       <c r="G11" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I11" s="16" t="s">
+      <c r="J11" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="J11" s="16" t="s">
+      <c r="K11" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="K11" s="18" t="s">
+      <c r="L11" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>23</v>
       </c>
@@ -1492,17 +1511,17 @@
       <c r="G12" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="I12" s="16" t="s">
+      <c r="J12" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="J12" s="16" t="s">
+      <c r="K12" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="K12" s="18" t="s">
+      <c r="L12" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>26</v>
       </c>
@@ -1521,17 +1540,17 @@
       <c r="G13" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I13" s="16" t="s">
+      <c r="J13" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="J13" s="16" t="s">
+      <c r="K13" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="K13" s="18" t="s">
+      <c r="L13" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>30</v>
       </c>
@@ -1550,17 +1569,17 @@
       <c r="G14" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="I14" s="16" t="s">
+      <c r="J14" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="J14" s="16" t="s">
+      <c r="K14" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="K14" s="18" t="s">
+      <c r="L14" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" s="22" t="s">
         <v>165</v>
       </c>
@@ -1579,17 +1598,17 @@
       <c r="G15" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="I15" s="16" t="s">
+      <c r="J15" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="J15" s="16" t="s">
+      <c r="K15" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="K15" s="18" t="s">
+      <c r="L15" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" s="22" t="s">
         <v>167</v>
       </c>
@@ -1608,17 +1627,17 @@
       <c r="G16" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="I16" s="16" t="s">
+      <c r="J16" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="J16" s="16" t="s">
+      <c r="K16" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="K16" s="18" t="s">
+      <c r="L16" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>32</v>
       </c>
@@ -1628,17 +1647,29 @@
       <c r="C17" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="I17" s="16" t="s">
+      <c r="E17" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>173</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="H17" t="s">
+        <v>171</v>
+      </c>
+      <c r="J17" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="J17" s="16" t="s">
+      <c r="K17" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="K17" s="18" t="s">
+      <c r="L17" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>34</v>
       </c>
@@ -1648,17 +1679,29 @@
       <c r="C18" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I18" s="20" t="s">
+      <c r="E18" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="H18" t="s">
+        <v>176</v>
+      </c>
+      <c r="J18" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="J18" s="20" t="s">
+      <c r="K18" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="K18" s="18" t="s">
+      <c r="L18" s="18" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" s="15" t="s">
         <v>36</v>
       </c>
@@ -1668,17 +1711,24 @@
       <c r="C19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I19" s="16" t="s">
+      <c r="E19" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="G19" s="1"/>
+      <c r="J19" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="J19" s="16" t="s">
+      <c r="K19" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="K19" s="18" t="s">
+      <c r="L19" s="18" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" s="13" t="s">
         <v>38</v>
       </c>
@@ -1688,17 +1738,24 @@
       <c r="C20" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I20" s="16" t="s">
+      <c r="E20" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="G20" s="1"/>
+      <c r="J20" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="J20" s="16" t="s">
+      <c r="K20" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="K20" s="18" t="s">
+      <c r="L20" s="18" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A21" s="25" t="s">
         <v>79</v>
       </c>
@@ -1708,17 +1765,24 @@
       <c r="C21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I21" s="16" t="s">
+      <c r="E21" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="G21" s="1"/>
+      <c r="J21" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="J21" s="16" t="s">
+      <c r="K21" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="K21" s="18" t="s">
+      <c r="L21" s="18" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>81</v>
       </c>
@@ -1728,17 +1792,24 @@
       <c r="C22" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I22" s="16" t="s">
+      <c r="E22" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="G22" s="1"/>
+      <c r="J22" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="J22" s="16" t="s">
+      <c r="K22" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="K22" s="18" t="s">
+      <c r="L22" s="18" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>83</v>
       </c>
@@ -1748,17 +1819,24 @@
       <c r="C23" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I23" s="16" t="s">
+      <c r="E23" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="G23" s="1"/>
+      <c r="J23" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="J23" s="16" t="s">
+      <c r="K23" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="K23" s="18" t="s">
+      <c r="L23" s="18" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>85</v>
       </c>
@@ -1768,17 +1846,24 @@
       <c r="C24" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I24" s="16" t="s">
+      <c r="E24" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="G24" s="1"/>
+      <c r="J24" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="J24" s="16" t="s">
+      <c r="K24" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="K24" s="18" t="s">
+      <c r="L24" s="18" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>87</v>
       </c>
@@ -1788,17 +1873,17 @@
       <c r="C25" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I25" s="16" t="s">
+      <c r="J25" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="J25" s="16" t="s">
+      <c r="K25" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="K25" s="18" t="s">
+      <c r="L25" s="18" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" s="23" t="s">
         <v>169</v>
       </c>
@@ -1808,205 +1893,205 @@
       <c r="C26" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="I26" s="16" t="s">
+      <c r="J26" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="J26" s="16" t="s">
+      <c r="K26" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="K26" s="18" t="s">
+      <c r="L26" s="18" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="I27" s="3" t="s">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="J27" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="J27" s="3" t="s">
+      <c r="K27" s="3" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="I28" s="3" t="s">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="J28" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="J28" s="3" t="s">
+      <c r="K28" s="3" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="I29" s="3" t="s">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="J29" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="J29" s="3" t="s">
+      <c r="K29" s="3" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="I30" s="3" t="s">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="J30" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="J30" s="3" t="s">
+      <c r="K30" s="3" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="I31" s="3" t="s">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="J31" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="J31" s="3" t="s">
+      <c r="K31" s="3" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="I32" s="3" t="s">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="J32" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="J32" s="3" t="s">
+      <c r="K32" s="3" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I33" s="3" t="s">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J33" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="J33" s="1" t="s">
+      <c r="K33" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I34" s="3" t="s">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J34" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J34" s="1" t="s">
+      <c r="K34" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I35" s="3" t="s">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J35" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="J35" s="1" t="s">
+      <c r="K35" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I36" s="3" t="s">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J36" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="J36" s="1" t="s">
+      <c r="K36" s="1" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I37" s="10" t="s">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J37" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="J37" s="10" t="s">
+      <c r="K37" s="10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I38" s="10" t="s">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J38" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="J38" s="10" t="s">
+      <c r="K38" s="10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I39" s="10" t="s">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J39" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="J39" s="10" t="s">
+      <c r="K39" s="10" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I40" s="10" t="s">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J40" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="J40" s="10" t="s">
+      <c r="K40" s="10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I41" s="10" t="s">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J41" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="J41" s="10" t="s">
+      <c r="K41" s="10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I42" s="10" t="s">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J42" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="J42" s="10" t="s">
+      <c r="K42" s="10" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I43" s="10" t="s">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J43" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="J43" s="10" t="s">
+      <c r="K43" s="10" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I44" s="10" t="s">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J44" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="J44" s="10" t="s">
+      <c r="K44" s="10" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I45" s="10" t="s">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J45" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="J45" s="10" t="s">
+      <c r="K45" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="9"/>
       <c r="B46" s="9"/>
-      <c r="I46" s="10" t="s">
+      <c r="J46" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="J46" s="10" t="s">
+      <c r="K46" s="10" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I47" s="10" t="s">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J47" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="J47" s="10" t="s">
+      <c r="K47" s="10" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="I48" s="10" t="s">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="J48" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="J48" s="10" t="s">
+      <c r="K48" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="49" spans="9:10" x14ac:dyDescent="0.35">
-      <c r="I49" s="10" t="s">
+    <row r="49" spans="10:11" x14ac:dyDescent="0.35">
+      <c r="J49" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="J49" s="10" t="s">
+      <c r="K49" s="10" t="s">
         <v>78</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="I1:K1"/>
+    <mergeCell ref="J1:L1"/>
     <mergeCell ref="E1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>